<commit_message>
Actualizar archivos de coloración y productos en formato Excel
</commit_message>
<xml_diff>
--- a/wella/coloracion.xlsx
+++ b/wella/coloracion.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="395">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="643" uniqueCount="402">
   <si>
     <t>Tono</t>
   </si>
@@ -936,21 +936,12 @@
     <t>CT PLUS 60ML 55/03 INT LIGHT BROWN NAT GOLD</t>
   </si>
   <si>
-    <t>CT PLUS 60ML 55/05 INT LIGHT-BR NAT MH</t>
-  </si>
-  <si>
     <t>CT PLUS 60ML 55/07 INT LIGHT BR NAT BROWN</t>
   </si>
   <si>
     <t>CT PLUS 60ML 66/03 INT DARK BL NAT GOLD</t>
   </si>
   <si>
-    <t>CT PLUS 60ML 66/04 INT DARK-BL NAT RED</t>
-  </si>
-  <si>
-    <t>CT PLUS 60ML 66/07 INT DARK BL NAT BR</t>
-  </si>
-  <si>
     <t>CT PLUS 60ML 77/07 INT MED BL NAT BR</t>
   </si>
   <si>
@@ -1204,6 +1195,36 @@
   </si>
   <si>
     <t>Linea</t>
+  </si>
+  <si>
+    <t>WP CT MP ATB PURE NAT 8/05 60ML LATAM</t>
+  </si>
+  <si>
+    <t>WP CT MP ATB PURE NAT 10/05 60ML LATAM</t>
+  </si>
+  <si>
+    <t>WP CT MP ATB PURE NAT 6/05 60ML LATAM</t>
+  </si>
+  <si>
+    <t>WP CT MP ATB DEEP BRN 8/73 60ML LATAM</t>
+  </si>
+  <si>
+    <t>WP CT MP ATB PURE NAT 10/0 60ML LATAM</t>
+  </si>
+  <si>
+    <t>WP CT MP ATB RICH NAT 10/6 60ML LATAM</t>
+  </si>
+  <si>
+    <t>WP CT MP ATB SPEC MIX 0/45 60ml LATAM</t>
+  </si>
+  <si>
+    <t>WP CT MP ATB VIB RED 8/43 60ML LATAM</t>
+  </si>
+  <si>
+    <t>WP CT MP ATB RICH NAT 9/16 60ML LATAM</t>
+  </si>
+  <si>
+    <t>WP CT MP ATB VIB RED 55/65 60ML LATAM</t>
   </si>
 </sst>
 </file>
@@ -1240,7 +1261,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1250,6 +1271,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1321,7 +1354,7 @@
       <alignment vertical="top"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1342,12 +1375,60 @@
       <alignment horizontal="left" vertical="top"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 105" xfId="1"/>
   </cellStyles>
-  <dxfs count="21">
+  <dxfs count="29">
+    <dxf>
+      <font>
+        <color theme="0" tint="-0.24994659260841701"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0" tint="-0.24994659260841701"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0" tint="-0.24994659260841701"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0" tint="-0.24994659260841701"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0" tint="-0.24994659260841701"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0" tint="-0.24994659260841701"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0" tint="-0.24994659260841701"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0" tint="-0.24994659260841701"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <color theme="0" tint="-0.24994659260841701"/>
@@ -1753,7 +1834,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C239"/>
+  <dimension ref="A1:C246"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.85546875" bestFit="1" customWidth="1"/>
@@ -1768,7 +1849,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -2672,8 +2753,8 @@
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A84" s="2" t="s">
-        <v>203</v>
+      <c r="A84" s="6" t="s">
+        <v>304</v>
       </c>
       <c r="B84" s="2" t="s">
         <v>255</v>
@@ -2683,8 +2764,8 @@
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A85" s="2" t="s">
-        <v>204</v>
+      <c r="A85" s="6" t="s">
+        <v>305</v>
       </c>
       <c r="B85" s="2" t="s">
         <v>256</v>
@@ -2694,8 +2775,8 @@
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A86" s="2" t="s">
-        <v>205</v>
+      <c r="A86" s="6" t="s">
+        <v>306</v>
       </c>
       <c r="B86" s="2" t="s">
         <v>257</v>
@@ -2705,8 +2786,8 @@
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A87" s="2" t="s">
-        <v>206</v>
+      <c r="A87" s="6" t="s">
+        <v>307</v>
       </c>
       <c r="B87" s="2" t="s">
         <v>258</v>
@@ -2717,7 +2798,7 @@
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
-        <v>207</v>
+        <v>308</v>
       </c>
       <c r="B88" s="2" t="s">
         <v>259</v>
@@ -2727,8 +2808,8 @@
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A89" s="2" t="s">
-        <v>208</v>
+      <c r="A89" s="6" t="s">
+        <v>309</v>
       </c>
       <c r="B89" s="2"/>
       <c r="C89" s="3" t="s">
@@ -2737,7 +2818,7 @@
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="B90" s="2"/>
       <c r="C90" s="3" t="s">
@@ -2745,8 +2826,8 @@
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A91" s="2" t="s">
-        <v>210</v>
+      <c r="A91" s="6" t="s">
+        <v>204</v>
       </c>
       <c r="B91" s="2" t="s">
         <v>260</v>
@@ -2757,7 +2838,7 @@
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="B92" s="2" t="s">
         <v>261</v>
@@ -2767,8 +2848,8 @@
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A93" s="2" t="s">
-        <v>212</v>
+      <c r="A93" s="6" t="s">
+        <v>206</v>
       </c>
       <c r="B93" s="2" t="s">
         <v>262</v>
@@ -2779,7 +2860,7 @@
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="B94" s="2"/>
       <c r="C94" s="3" t="s">
@@ -2787,8 +2868,8 @@
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A95" s="2" t="s">
-        <v>214</v>
+      <c r="A95" s="7" t="s">
+        <v>208</v>
       </c>
       <c r="B95" s="2" t="s">
         <v>263</v>
@@ -2798,8 +2879,8 @@
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A96" s="2" t="s">
-        <v>215</v>
+      <c r="A96" s="6" t="s">
+        <v>209</v>
       </c>
       <c r="B96" s="2" t="s">
         <v>264</v>
@@ -2809,8 +2890,8 @@
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A97" s="2" t="s">
-        <v>216</v>
+      <c r="A97" s="6" t="s">
+        <v>210</v>
       </c>
       <c r="B97" s="2" t="s">
         <v>265</v>
@@ -2820,8 +2901,8 @@
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A98" s="2" t="s">
-        <v>217</v>
+      <c r="A98" s="6" t="s">
+        <v>211</v>
       </c>
       <c r="B98" s="2" t="s">
         <v>266</v>
@@ -2831,8 +2912,8 @@
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A99" s="2" t="s">
-        <v>218</v>
+      <c r="A99" s="6" t="s">
+        <v>212</v>
       </c>
       <c r="B99" s="2" t="s">
         <v>267</v>
@@ -2842,8 +2923,8 @@
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A100" s="2" t="s">
-        <v>219</v>
+      <c r="A100" s="7" t="s">
+        <v>213</v>
       </c>
       <c r="B100" s="2" t="s">
         <v>268</v>
@@ -2853,8 +2934,8 @@
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A101" s="2" t="s">
-        <v>220</v>
+      <c r="A101" s="6" t="s">
+        <v>214</v>
       </c>
       <c r="B101" s="2" t="s">
         <v>269</v>
@@ -2865,7 +2946,7 @@
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="B102" s="2" t="s">
         <v>270</v>
@@ -2875,8 +2956,8 @@
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A103" s="2" t="s">
-        <v>222</v>
+      <c r="A103" s="6" t="s">
+        <v>216</v>
       </c>
       <c r="B103" s="2" t="s">
         <v>271</v>
@@ -2886,8 +2967,8 @@
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A104" s="2" t="s">
-        <v>223</v>
+      <c r="A104" s="6" t="s">
+        <v>217</v>
       </c>
       <c r="B104" s="2" t="s">
         <v>272</v>
@@ -2897,8 +2978,8 @@
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A105" s="2" t="s">
-        <v>224</v>
+      <c r="A105" s="6" t="s">
+        <v>218</v>
       </c>
       <c r="B105" s="2" t="s">
         <v>273</v>
@@ -2908,8 +2989,8 @@
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A106" s="2" t="s">
-        <v>225</v>
+      <c r="A106" s="7" t="s">
+        <v>219</v>
       </c>
       <c r="B106" s="2" t="s">
         <v>274</v>
@@ -2919,8 +3000,8 @@
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A107" s="2" t="s">
-        <v>226</v>
+      <c r="A107" s="6" t="s">
+        <v>220</v>
       </c>
       <c r="B107" s="2" t="s">
         <v>275</v>
@@ -2931,7 +3012,7 @@
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="B108" s="2" t="s">
         <v>276</v>
@@ -2941,8 +3022,8 @@
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A109" s="2" t="s">
-        <v>228</v>
+      <c r="A109" s="6" t="s">
+        <v>222</v>
       </c>
       <c r="B109" s="2" t="s">
         <v>277</v>
@@ -2952,8 +3033,8 @@
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A110" s="2" t="s">
-        <v>229</v>
+      <c r="A110" s="7" t="s">
+        <v>223</v>
       </c>
       <c r="B110" s="2" t="s">
         <v>278</v>
@@ -2964,7 +3045,7 @@
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="B111" s="2" t="s">
         <v>279</v>
@@ -2975,7 +3056,7 @@
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="B112" s="2" t="s">
         <v>280</v>
@@ -2985,8 +3066,8 @@
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A113" s="2" t="s">
-        <v>232</v>
+      <c r="A113" s="6" t="s">
+        <v>226</v>
       </c>
       <c r="B113" s="2" t="s">
         <v>281</v>
@@ -2996,8 +3077,8 @@
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A114" s="2" t="s">
-        <v>233</v>
+      <c r="A114" s="6" t="s">
+        <v>227</v>
       </c>
       <c r="B114" s="2" t="s">
         <v>282</v>
@@ -3007,8 +3088,8 @@
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A115" s="2" t="s">
-        <v>234</v>
+      <c r="A115" s="6" t="s">
+        <v>228</v>
       </c>
       <c r="B115" s="2" t="s">
         <v>283</v>
@@ -3019,7 +3100,7 @@
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="B116" s="2" t="s">
         <v>284</v>
@@ -3030,7 +3111,7 @@
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="B117" s="2" t="s">
         <v>285</v>
@@ -3041,7 +3122,7 @@
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="B118" s="2" t="s">
         <v>286</v>
@@ -3051,8 +3132,8 @@
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A119" s="2" t="s">
-        <v>238</v>
+      <c r="A119" s="6" t="s">
+        <v>232</v>
       </c>
       <c r="B119" s="2" t="s">
         <v>287</v>
@@ -3062,8 +3143,8 @@
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A120" s="2" t="s">
-        <v>239</v>
+      <c r="A120" s="6" t="s">
+        <v>233</v>
       </c>
       <c r="B120" s="2" t="s">
         <v>288</v>
@@ -3073,8 +3154,8 @@
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A121" s="2" t="s">
-        <v>240</v>
+      <c r="A121" s="6" t="s">
+        <v>234</v>
       </c>
       <c r="B121" s="2" t="s">
         <v>289</v>
@@ -3084,8 +3165,8 @@
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A122" s="2" t="s">
-        <v>241</v>
+      <c r="A122" s="6" t="s">
+        <v>235</v>
       </c>
       <c r="B122" s="2" t="s">
         <v>290</v>
@@ -3096,7 +3177,7 @@
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="B123" s="2" t="s">
         <v>291</v>
@@ -3107,7 +3188,7 @@
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="B124" s="2" t="s">
         <v>292</v>
@@ -3117,8 +3198,8 @@
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A125" s="2" t="s">
-        <v>244</v>
+      <c r="A125" s="6" t="s">
+        <v>238</v>
       </c>
       <c r="B125" s="2" t="s">
         <v>293</v>
@@ -3129,7 +3210,7 @@
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="B126" s="2" t="s">
         <v>294</v>
@@ -3139,8 +3220,8 @@
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A127" s="2" t="s">
-        <v>246</v>
+      <c r="A127" s="6" t="s">
+        <v>240</v>
       </c>
       <c r="B127" s="2" t="s">
         <v>295</v>
@@ -3150,8 +3231,8 @@
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A128" s="2" t="s">
-        <v>247</v>
+      <c r="A128" s="7" t="s">
+        <v>241</v>
       </c>
       <c r="B128" s="2" t="s">
         <v>296</v>
@@ -3161,8 +3242,8 @@
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A129" s="2" t="s">
-        <v>248</v>
+      <c r="A129" s="6" t="s">
+        <v>242</v>
       </c>
       <c r="B129" s="2" t="s">
         <v>297</v>
@@ -3173,7 +3254,7 @@
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="B130" s="2" t="s">
         <v>298</v>
@@ -3184,7 +3265,7 @@
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="B131" s="2" t="s">
         <v>299</v>
@@ -3194,8 +3275,8 @@
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A132" s="2" t="s">
-        <v>251</v>
+      <c r="A132" s="6" t="s">
+        <v>245</v>
       </c>
       <c r="B132" s="2" t="s">
         <v>300</v>
@@ -3205,8 +3286,8 @@
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A133" s="2" t="s">
-        <v>252</v>
+      <c r="A133" s="6" t="s">
+        <v>246</v>
       </c>
       <c r="B133" s="2" t="s">
         <v>301</v>
@@ -3216,8 +3297,8 @@
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A134" s="2" t="s">
-        <v>253</v>
+      <c r="A134" s="6" t="s">
+        <v>247</v>
       </c>
       <c r="B134" s="2" t="s">
         <v>302</v>
@@ -3227,8 +3308,8 @@
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A135" s="5" t="s">
-        <v>254</v>
+      <c r="A135" s="6" t="s">
+        <v>248</v>
       </c>
       <c r="B135" s="5" t="s">
         <v>303</v>
@@ -3238,8 +3319,8 @@
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A136" s="2" t="s">
-        <v>304</v>
+      <c r="A136" s="6" t="s">
+        <v>249</v>
       </c>
       <c r="B136" s="2">
         <v>5503</v>
@@ -3249,8 +3330,8 @@
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A137" s="2" t="s">
-        <v>305</v>
+      <c r="A137" s="6" t="s">
+        <v>250</v>
       </c>
       <c r="B137" s="2">
         <v>5505</v>
@@ -3260,8 +3341,8 @@
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A138" s="2" t="s">
-        <v>306</v>
+      <c r="A138" s="6" t="s">
+        <v>251</v>
       </c>
       <c r="B138" s="2"/>
       <c r="C138" s="3" t="s">
@@ -3269,8 +3350,8 @@
       </c>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A139" s="2" t="s">
-        <v>307</v>
+      <c r="A139" s="6" t="s">
+        <v>252</v>
       </c>
       <c r="B139" s="2">
         <v>6603</v>
@@ -3281,7 +3362,7 @@
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
-        <v>308</v>
+        <v>253</v>
       </c>
       <c r="B140" s="2">
         <v>6604</v>
@@ -3291,572 +3372,556 @@
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A141" s="2" t="s">
-        <v>309</v>
-      </c>
-      <c r="B141" s="2">
+      <c r="A141" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="B141" s="2"/>
+      <c r="C141" s="3" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A142" s="6" t="s">
+        <v>392</v>
+      </c>
+      <c r="B142" s="2"/>
+      <c r="C142" s="3" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A143" s="6" t="s">
+        <v>393</v>
+      </c>
+      <c r="B143" s="2"/>
+      <c r="C143" s="3" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A144" s="6" t="s">
+        <v>394</v>
+      </c>
+      <c r="B144" s="2"/>
+      <c r="C144" s="3" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A145" s="6" t="s">
+        <v>395</v>
+      </c>
+      <c r="B145" s="2"/>
+      <c r="C145" s="3" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A146" s="6" t="s">
+        <v>396</v>
+      </c>
+      <c r="B146" s="2">
         <v>6607</v>
       </c>
-      <c r="C141" s="3" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A142" s="2" t="s">
-        <v>310</v>
-      </c>
-      <c r="B142" s="2">
+      <c r="C146" s="3" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A147" s="6" t="s">
+        <v>397</v>
+      </c>
+      <c r="B147" s="2"/>
+      <c r="C147" s="3" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A148" s="6" t="s">
+        <v>398</v>
+      </c>
+      <c r="B148" s="2"/>
+      <c r="C148" s="3" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A149" s="6" t="s">
+        <v>399</v>
+      </c>
+      <c r="B149" s="2"/>
+      <c r="C149" s="3" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A150" s="6" t="s">
+        <v>400</v>
+      </c>
+      <c r="B150" s="2">
         <v>7707</v>
       </c>
-      <c r="C142" s="3" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A143" s="2" t="s">
-        <v>311</v>
-      </c>
-      <c r="B143" s="2">
+      <c r="C150" s="3" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A151" s="6" t="s">
+        <v>401</v>
+      </c>
+      <c r="B151" s="2">
         <v>8803</v>
       </c>
-      <c r="C143" s="3" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A144" s="2" t="s">
-        <v>312</v>
-      </c>
-      <c r="B144" s="2">
-        <v>8807</v>
-      </c>
-      <c r="C144" s="3" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A145" s="2" t="s">
-        <v>314</v>
-      </c>
-      <c r="B145" s="2" t="s">
-        <v>354</v>
-      </c>
-      <c r="C145" s="3" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A146" s="2" t="s">
-        <v>315</v>
-      </c>
-      <c r="B146" s="2" t="s">
-        <v>355</v>
-      </c>
-      <c r="C146" s="3" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A147" s="2" t="s">
-        <v>316</v>
-      </c>
-      <c r="B147" s="2" t="s">
-        <v>356</v>
-      </c>
-      <c r="C147" s="3" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A148" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="B148" s="2" t="s">
-        <v>357</v>
-      </c>
-      <c r="C148" s="3" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A149" s="2" t="s">
-        <v>318</v>
-      </c>
-      <c r="B149" s="2" t="s">
-        <v>358</v>
-      </c>
-      <c r="C149" s="3" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A150" s="2" t="s">
-        <v>319</v>
-      </c>
-      <c r="B150" s="2" t="s">
-        <v>359</v>
-      </c>
-      <c r="C150" s="3" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A151" s="2" t="s">
-        <v>320</v>
-      </c>
-      <c r="B151" s="2" t="s">
-        <v>360</v>
-      </c>
       <c r="C151" s="3" t="s">
-        <v>313</v>
+        <v>202</v>
       </c>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
-        <v>321</v>
+        <v>311</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>361</v>
+        <v>351</v>
       </c>
       <c r="C152" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
-        <v>322</v>
+        <v>312</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>362</v>
+        <v>352</v>
       </c>
       <c r="C153" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
-        <v>323</v>
+        <v>313</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>363</v>
+        <v>353</v>
       </c>
       <c r="C154" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A155" s="2" t="s">
-        <v>324</v>
+        <v>314</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>364</v>
+        <v>354</v>
       </c>
       <c r="C155" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
-        <v>325</v>
+        <v>315</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>365</v>
+        <v>355</v>
       </c>
       <c r="C156" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A157" s="2" t="s">
-        <v>326</v>
+        <v>316</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>366</v>
+        <v>356</v>
       </c>
       <c r="C157" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
-        <v>327</v>
+        <v>317</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>367</v>
+        <v>357</v>
       </c>
       <c r="C158" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
-        <v>328</v>
+        <v>318</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>368</v>
+        <v>358</v>
       </c>
       <c r="C159" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
-        <v>329</v>
+        <v>319</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>369</v>
+        <v>359</v>
       </c>
       <c r="C160" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
-        <v>330</v>
+        <v>320</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>370</v>
+        <v>360</v>
       </c>
       <c r="C161" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
-        <v>331</v>
+        <v>321</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>371</v>
+        <v>361</v>
       </c>
       <c r="C162" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A163" s="2" t="s">
-        <v>332</v>
+        <v>322</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>372</v>
+        <v>362</v>
       </c>
       <c r="C163" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A164" s="2" t="s">
-        <v>333</v>
+        <v>323</v>
       </c>
       <c r="B164" s="2" t="s">
-        <v>373</v>
+        <v>363</v>
       </c>
       <c r="C164" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A165" s="2" t="s">
-        <v>334</v>
+        <v>324</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>374</v>
+        <v>364</v>
       </c>
       <c r="C165" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A166" s="2" t="s">
-        <v>335</v>
+        <v>325</v>
       </c>
       <c r="B166" s="2" t="s">
-        <v>375</v>
+        <v>365</v>
       </c>
       <c r="C166" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A167" s="2" t="s">
-        <v>336</v>
+        <v>326</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>376</v>
+        <v>366</v>
       </c>
       <c r="C167" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A168" s="2" t="s">
-        <v>337</v>
+        <v>327</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>377</v>
+        <v>367</v>
       </c>
       <c r="C168" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A169" s="2" t="s">
-        <v>338</v>
+        <v>328</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>378</v>
+        <v>368</v>
       </c>
       <c r="C169" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A170" s="2" t="s">
-        <v>339</v>
+        <v>329</v>
       </c>
       <c r="B170" s="2" t="s">
-        <v>379</v>
+        <v>369</v>
       </c>
       <c r="C170" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A171" s="2" t="s">
-        <v>340</v>
+        <v>330</v>
       </c>
       <c r="B171" s="2" t="s">
-        <v>380</v>
+        <v>370</v>
       </c>
       <c r="C171" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A172" s="2" t="s">
-        <v>341</v>
+        <v>331</v>
       </c>
       <c r="B172" s="2" t="s">
-        <v>381</v>
+        <v>371</v>
       </c>
       <c r="C172" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A173" s="2" t="s">
-        <v>342</v>
+        <v>332</v>
       </c>
       <c r="B173" s="2" t="s">
-        <v>382</v>
+        <v>372</v>
       </c>
       <c r="C173" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A174" s="2" t="s">
-        <v>343</v>
+        <v>333</v>
       </c>
       <c r="B174" s="2" t="s">
-        <v>383</v>
+        <v>373</v>
       </c>
       <c r="C174" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A175" s="2" t="s">
-        <v>344</v>
+        <v>334</v>
       </c>
       <c r="B175" s="2" t="s">
-        <v>384</v>
+        <v>374</v>
       </c>
       <c r="C175" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A176" s="2" t="s">
-        <v>345</v>
+        <v>335</v>
       </c>
       <c r="B176" s="2" t="s">
-        <v>385</v>
+        <v>375</v>
       </c>
       <c r="C176" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177" s="2" t="s">
-        <v>346</v>
+        <v>336</v>
       </c>
       <c r="B177" s="2" t="s">
-        <v>386</v>
+        <v>376</v>
       </c>
       <c r="C177" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A178" s="2" t="s">
-        <v>347</v>
+        <v>337</v>
       </c>
       <c r="B178" s="2" t="s">
-        <v>387</v>
+        <v>377</v>
       </c>
       <c r="C178" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A179" s="2" t="s">
-        <v>348</v>
+        <v>338</v>
       </c>
       <c r="B179" s="2" t="s">
-        <v>388</v>
+        <v>378</v>
       </c>
       <c r="C179" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A180" s="2" t="s">
-        <v>349</v>
+        <v>339</v>
       </c>
       <c r="B180" s="2" t="s">
-        <v>389</v>
+        <v>379</v>
       </c>
       <c r="C180" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A181" s="2" t="s">
-        <v>350</v>
+        <v>340</v>
       </c>
       <c r="B181" s="2" t="s">
-        <v>390</v>
+        <v>380</v>
       </c>
       <c r="C181" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A182" s="2" t="s">
-        <v>351</v>
+        <v>341</v>
       </c>
       <c r="B182" s="2" t="s">
-        <v>391</v>
+        <v>381</v>
       </c>
       <c r="C182" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A183" s="2" t="s">
-        <v>352</v>
+        <v>342</v>
       </c>
       <c r="B183" s="2" t="s">
-        <v>392</v>
+        <v>382</v>
       </c>
       <c r="C183" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A184" s="2" t="s">
-        <v>353</v>
+        <v>343</v>
       </c>
       <c r="B184" s="2" t="s">
-        <v>393</v>
+        <v>383</v>
       </c>
       <c r="C184" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A185" s="2" t="s">
-        <v>2</v>
+        <v>344</v>
       </c>
       <c r="B185" s="2" t="s">
-        <v>57</v>
+        <v>384</v>
       </c>
       <c r="C185" s="3" t="s">
-        <v>112</v>
+        <v>310</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A186" s="2" t="s">
-        <v>3</v>
+        <v>345</v>
       </c>
       <c r="B186" s="2" t="s">
-        <v>58</v>
+        <v>385</v>
       </c>
       <c r="C186" s="3" t="s">
-        <v>112</v>
+        <v>310</v>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A187" s="2" t="s">
-        <v>4</v>
+        <v>346</v>
       </c>
       <c r="B187" s="2" t="s">
-        <v>59</v>
+        <v>386</v>
       </c>
       <c r="C187" s="3" t="s">
-        <v>112</v>
+        <v>310</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A188" s="2" t="s">
-        <v>5</v>
+        <v>347</v>
       </c>
       <c r="B188" s="2" t="s">
-        <v>60</v>
+        <v>387</v>
       </c>
       <c r="C188" s="3" t="s">
-        <v>112</v>
+        <v>310</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A189" s="2" t="s">
-        <v>6</v>
+        <v>348</v>
       </c>
       <c r="B189" s="2" t="s">
-        <v>61</v>
+        <v>388</v>
       </c>
       <c r="C189" s="3" t="s">
-        <v>112</v>
+        <v>310</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A190" s="2" t="s">
-        <v>7</v>
+        <v>349</v>
       </c>
       <c r="B190" s="2" t="s">
-        <v>62</v>
+        <v>389</v>
       </c>
       <c r="C190" s="3" t="s">
-        <v>112</v>
+        <v>310</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A191" s="2" t="s">
-        <v>8</v>
+        <v>350</v>
       </c>
       <c r="B191" s="2" t="s">
-        <v>63</v>
+        <v>390</v>
       </c>
       <c r="C191" s="3" t="s">
-        <v>112</v>
+        <v>310</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A192" s="2" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="B192" s="2" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="C192" s="3" t="s">
         <v>112</v>
@@ -3864,10 +3929,10 @@
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A193" s="2" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B193" s="2" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="C193" s="3" t="s">
         <v>112</v>
@@ -3875,10 +3940,10 @@
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A194" s="2" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="B194" s="2" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="C194" s="3" t="s">
         <v>112</v>
@@ -3886,10 +3951,10 @@
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A195" s="2" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="B195" s="2" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="C195" s="3" t="s">
         <v>112</v>
@@ -3897,10 +3962,10 @@
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A196" s="2" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="B196" s="2" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="C196" s="3" t="s">
         <v>112</v>
@@ -3908,10 +3973,10 @@
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A197" s="2" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B197" s="2" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="C197" s="3" t="s">
         <v>112</v>
@@ -3919,10 +3984,10 @@
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A198" s="2" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B198" s="2" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="C198" s="3" t="s">
         <v>112</v>
@@ -3930,10 +3995,10 @@
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A199" s="2" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="B199" s="2" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="C199" s="3" t="s">
         <v>112</v>
@@ -3941,10 +4006,10 @@
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A200" s="2" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="B200" s="2" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="C200" s="3" t="s">
         <v>112</v>
@@ -3952,10 +4017,10 @@
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A201" s="2" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="B201" s="2" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="C201" s="3" t="s">
         <v>112</v>
@@ -3963,10 +4028,10 @@
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A202" s="2" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="B202" s="2" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="C202" s="3" t="s">
         <v>112</v>
@@ -3974,10 +4039,10 @@
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A203" s="2" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="B203" s="2" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="C203" s="3" t="s">
         <v>112</v>
@@ -3985,10 +4050,10 @@
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A204" s="2" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="B204" s="2" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="C204" s="3" t="s">
         <v>112</v>
@@ -3996,10 +4061,10 @@
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A205" s="2" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="B205" s="2" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="C205" s="3" t="s">
         <v>112</v>
@@ -4007,10 +4072,10 @@
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A206" s="2" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="B206" s="2" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="C206" s="3" t="s">
         <v>112</v>
@@ -4018,10 +4083,10 @@
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A207" s="2" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B207" s="2" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="C207" s="3" t="s">
         <v>112</v>
@@ -4029,10 +4094,10 @@
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A208" s="2" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="B208" s="2" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="C208" s="3" t="s">
         <v>112</v>
@@ -4040,10 +4105,10 @@
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A209" s="2" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="B209" s="2" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="C209" s="3" t="s">
         <v>112</v>
@@ -4051,10 +4116,10 @@
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A210" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B210" s="2" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="C210" s="3" t="s">
         <v>112</v>
@@ -4062,10 +4127,10 @@
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A211" s="2" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="B211" s="2" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="C211" s="3" t="s">
         <v>112</v>
@@ -4073,10 +4138,10 @@
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A212" s="2" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="B212" s="2" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="C212" s="3" t="s">
         <v>112</v>
@@ -4084,10 +4149,10 @@
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A213" s="2" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="B213" s="2" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="C213" s="3" t="s">
         <v>112</v>
@@ -4095,10 +4160,10 @@
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A214" s="2" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="B214" s="2" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="C214" s="3" t="s">
         <v>112</v>
@@ -4106,10 +4171,10 @@
     </row>
     <row r="215" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A215" s="2" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="B215" s="2" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="C215" s="3" t="s">
         <v>112</v>
@@ -4117,10 +4182,10 @@
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A216" s="2" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B216" s="2" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="C216" s="3" t="s">
         <v>112</v>
@@ -4128,10 +4193,10 @@
     </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A217" s="2" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B217" s="2" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="C217" s="3" t="s">
         <v>112</v>
@@ -4139,10 +4204,10 @@
     </row>
     <row r="218" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A218" s="2" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="B218" s="2" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="C218" s="3" t="s">
         <v>112</v>
@@ -4150,10 +4215,10 @@
     </row>
     <row r="219" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A219" s="2" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B219" s="2" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="C219" s="3" t="s">
         <v>112</v>
@@ -4161,10 +4226,10 @@
     </row>
     <row r="220" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A220" s="2" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="B220" s="2" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="C220" s="3" t="s">
         <v>112</v>
@@ -4172,10 +4237,10 @@
     </row>
     <row r="221" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A221" s="2" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="B221" s="2" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="C221" s="3" t="s">
         <v>112</v>
@@ -4183,10 +4248,10 @@
     </row>
     <row r="222" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A222" s="2" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="B222" s="2" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="C222" s="3" t="s">
         <v>112</v>
@@ -4194,10 +4259,10 @@
     </row>
     <row r="223" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A223" s="2" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="B223" s="2" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="C223" s="3" t="s">
         <v>112</v>
@@ -4205,10 +4270,10 @@
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A224" s="2" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="B224" s="2" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="C224" s="3" t="s">
         <v>112</v>
@@ -4216,10 +4281,10 @@
     </row>
     <row r="225" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A225" s="2" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="B225" s="2" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="C225" s="3" t="s">
         <v>112</v>
@@ -4227,10 +4292,10 @@
     </row>
     <row r="226" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A226" s="2" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="B226" s="2" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="C226" s="3" t="s">
         <v>112</v>
@@ -4238,10 +4303,10 @@
     </row>
     <row r="227" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A227" s="2" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="B227" s="2" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="C227" s="3" t="s">
         <v>112</v>
@@ -4249,10 +4314,10 @@
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A228" s="2" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="B228" s="2" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="C228" s="3" t="s">
         <v>112</v>
@@ -4260,10 +4325,10 @@
     </row>
     <row r="229" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A229" s="2" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="B229" s="2" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="C229" s="3" t="s">
         <v>112</v>
@@ -4271,10 +4336,10 @@
     </row>
     <row r="230" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A230" s="2" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="B230" s="2" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="C230" s="3" t="s">
         <v>112</v>
@@ -4282,10 +4347,10 @@
     </row>
     <row r="231" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A231" s="2" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="B231" s="2" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="C231" s="3" t="s">
         <v>112</v>
@@ -4293,10 +4358,10 @@
     </row>
     <row r="232" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A232" s="2" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="B232" s="2" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="C232" s="3" t="s">
         <v>112</v>
@@ -4304,10 +4369,10 @@
     </row>
     <row r="233" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A233" s="2" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="B233" s="2" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="C233" s="3" t="s">
         <v>112</v>
@@ -4315,10 +4380,10 @@
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A234" s="2" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="B234" s="2" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="C234" s="3" t="s">
         <v>112</v>
@@ -4326,10 +4391,10 @@
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A235" s="2" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="B235" s="2" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="C235" s="3" t="s">
         <v>112</v>
@@ -4337,10 +4402,10 @@
     </row>
     <row r="236" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A236" s="2" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B236" s="2" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="C236" s="3" t="s">
         <v>112</v>
@@ -4348,10 +4413,10 @@
     </row>
     <row r="237" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A237" s="2" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="B237" s="2" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="C237" s="3" t="s">
         <v>112</v>
@@ -4359,10 +4424,10 @@
     </row>
     <row r="238" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A238" s="2" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="B238" s="2" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="C238" s="3" t="s">
         <v>112</v>
@@ -4370,118 +4435,195 @@
     </row>
     <row r="239" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A239" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B239" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C239" s="3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="240" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A240" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B240" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C240" s="3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="241" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A241" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B241" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C241" s="3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="242" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A242" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B242" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C242" s="3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="243" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A243" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B243" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C243" s="3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="244" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A244" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B244" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C244" s="3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="245" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A245" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B245" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C245" s="3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="246" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A246" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B239" s="2" t="s">
+      <c r="B246" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="C239" s="3" t="s">
+      <c r="C246" s="3" t="s">
         <v>112</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A185:A239">
-    <cfRule type="expression" dxfId="20" priority="26">
+  <conditionalFormatting sqref="A192:A246">
+    <cfRule type="expression" dxfId="24" priority="29">
       <formula>#REF!="SIN STOCK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B185:B239">
-    <cfRule type="expression" dxfId="19" priority="25">
+  <conditionalFormatting sqref="B192:B246">
+    <cfRule type="expression" dxfId="23" priority="28">
       <formula>#REF!="SIN STOCK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C185">
-    <cfRule type="expression" dxfId="18" priority="24">
+  <conditionalFormatting sqref="C192">
+    <cfRule type="expression" dxfId="22" priority="27">
       <formula>#REF!="SIN STOCK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C186:C239">
-    <cfRule type="expression" dxfId="17" priority="23">
+  <conditionalFormatting sqref="C193:C246">
+    <cfRule type="expression" dxfId="21" priority="26">
       <formula>#REF!="SIN STOCK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:A71">
-    <cfRule type="expression" dxfId="16" priority="21">
+    <cfRule type="expression" dxfId="20" priority="24">
       <formula>#REF!="SIN STOCK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A73:A83">
-    <cfRule type="expression" dxfId="15" priority="20">
+    <cfRule type="expression" dxfId="19" priority="23">
       <formula>#REF!="SIN STOCK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:B71">
-    <cfRule type="expression" dxfId="14" priority="19">
+    <cfRule type="expression" dxfId="18" priority="22">
       <formula>#REF!="SIN STOCK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B73:B83">
-    <cfRule type="expression" dxfId="13" priority="18">
+    <cfRule type="expression" dxfId="17" priority="21">
       <formula>#REF!="SIN STOCK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:C83">
-    <cfRule type="expression" dxfId="12" priority="17">
+    <cfRule type="expression" dxfId="16" priority="20">
       <formula>#REF!="SIN STOCK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A135">
-    <cfRule type="expression" dxfId="11" priority="16">
-      <formula>#REF!="SIN STOCK"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A84:A134">
-    <cfRule type="expression" dxfId="10" priority="15">
+  <conditionalFormatting sqref="C84:C135">
+    <cfRule type="expression" dxfId="14" priority="15">
       <formula>#REF!="SIN STOCK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B135">
-    <cfRule type="expression" dxfId="9" priority="14">
+    <cfRule type="expression" dxfId="13" priority="17">
       <formula>#REF!="SIN STOCK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B84:B134">
-    <cfRule type="expression" dxfId="8" priority="13">
+    <cfRule type="expression" dxfId="12" priority="16">
       <formula>#REF!="SIN STOCK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C84:C135">
-    <cfRule type="expression" dxfId="7" priority="12">
+  <conditionalFormatting sqref="B136:B151">
+    <cfRule type="expression" dxfId="9" priority="13">
       <formula>#REF!="SIN STOCK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A136:A144">
-    <cfRule type="expression" dxfId="6" priority="11">
-      <formula>#REF!="SIN STOCK"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B136:B144">
-    <cfRule type="expression" dxfId="5" priority="10">
-      <formula>#REF!="SIN STOCK"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C136:C144">
-    <cfRule type="expression" dxfId="4" priority="9">
+  <conditionalFormatting sqref="C136:C151">
+    <cfRule type="expression" dxfId="8" priority="12">
       <formula>#REF!="SIN STOCK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A72">
-    <cfRule type="expression" dxfId="3" priority="6">
+    <cfRule type="expression" dxfId="7" priority="9">
       <formula>#REF!="SIN STOCK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A145:A184">
-    <cfRule type="expression" dxfId="2" priority="3">
+  <conditionalFormatting sqref="A152:A191">
+    <cfRule type="expression" dxfId="6" priority="6">
       <formula>#REF!="SIN STOCK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B145:B184">
-    <cfRule type="expression" dxfId="1" priority="2">
+  <conditionalFormatting sqref="B152:B191">
+    <cfRule type="expression" dxfId="5" priority="5">
       <formula>#REF!="SIN STOCK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C145:C184">
-    <cfRule type="expression" dxfId="0" priority="1">
+  <conditionalFormatting sqref="C152:C191">
+    <cfRule type="expression" dxfId="4" priority="4">
+      <formula>#REF!="SIN STOCK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A84:A140">
+    <cfRule type="expression" dxfId="3" priority="3">
+      <formula>#REF!="SIN STOCK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A141">
+    <cfRule type="expression" dxfId="2" priority="2">
+      <formula>#REF!="SIN STOCK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A142:A151">
+    <cfRule type="expression" dxfId="1" priority="1">
       <formula>#REF!="SIN STOCK"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>